<commit_message>
implement the demand change
demand change functionality was implemented in main.py
</commit_message>
<xml_diff>
--- a/data/scenarios.xlsx
+++ b/data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b9f352ed9e5ec6ce/00_플랜잇_철강inputoutput연구/steel_iotable/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{84D30074-6CA2-9646-BF7A-0F0212785F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85D9B1DD-4EF9-0D45-A43D-90390B00B298}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{84D30074-6CA2-9646-BF7A-0F0212785F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49A6F563-1CBE-564A-97B8-3D9CC85EB1D4}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="840" windowWidth="29400" windowHeight="17020" xr2:uid="{8A7290D0-0CEE-BE47-A4B5-AA6B65E25749}"/>
+    <workbookView xWindow="0" yWindow="840" windowWidth="29400" windowHeight="17020" xr2:uid="{8A7290D0-0CEE-BE47-A4B5-AA6B65E25749}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="10">
   <si>
     <t>sector</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>total</t>
+  </si>
+  <si>
+    <t>4506</t>
   </si>
 </sst>
 </file>
@@ -128,9 +131,9 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -146,6 +149,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -563,85 +570,85 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="4">
         <v>2711</v>
       </c>
-      <c r="C2" s="3">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3">
+      <c r="C2" s="2">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2">
         <v>-636028484.40622115</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <v>-1161255514.8874223</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="2">
         <v>-1161255514.8874218</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="2">
         <v>-1371346348.3328123</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="2">
         <v>-3152149612.6058397</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="2">
         <v>-3152149612.6058412</v>
       </c>
-      <c r="J2" s="3">
+      <c r="J2" s="2">
         <v>-3152149612.6058412</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="2">
         <v>-4145573278.2804456</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="2">
         <v>-4145573278.2804456</v>
       </c>
-      <c r="M2" s="3">
+      <c r="M2" s="2">
         <v>-5403129098.4650421</v>
       </c>
-      <c r="N2" s="3">
+      <c r="N2" s="2">
         <v>-6228563983.9188652</v>
       </c>
-      <c r="O2" s="3">
+      <c r="O2" s="2">
         <v>-6950163944.3933878</v>
       </c>
-      <c r="P2" s="3">
+      <c r="P2" s="2">
         <v>-6950163944.3933878</v>
       </c>
-      <c r="Q2" s="3">
+      <c r="Q2" s="2">
         <v>-6950163944.3933878</v>
       </c>
-      <c r="R2" s="3">
+      <c r="R2" s="2">
         <v>-7583661513.6934519</v>
       </c>
-      <c r="S2" s="3">
+      <c r="S2" s="2">
         <v>-7583661513.6934519</v>
       </c>
-      <c r="T2" s="3">
+      <c r="T2" s="2">
         <v>-8282886292.5491648</v>
       </c>
-      <c r="U2" s="3">
+      <c r="U2" s="2">
         <v>-8282886292.5491648</v>
       </c>
-      <c r="V2" s="3">
+      <c r="V2" s="2">
         <v>-8947849131.3262768</v>
       </c>
-      <c r="W2" s="3">
+      <c r="W2" s="2">
         <v>-8947849131.3262768</v>
       </c>
-      <c r="X2" s="3">
+      <c r="X2" s="2">
         <v>-9514046338.6238899</v>
       </c>
-      <c r="Y2" s="3">
+      <c r="Y2" s="2">
         <v>-9514046338.6238899</v>
       </c>
-      <c r="Z2" s="3">
+      <c r="Z2" s="2">
         <v>-9514046338.6238899</v>
       </c>
-      <c r="AA2" s="3">
+      <c r="AA2" s="2">
         <v>-9514046338.6238899</v>
       </c>
-      <c r="AB2" s="3">
+      <c r="AB2" s="2">
         <v>-9514046338.6238899</v>
       </c>
     </row>
@@ -649,85 +656,85 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
-        <v>4506</v>
-      </c>
-      <c r="C3" s="3">
+      <c r="B3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2">
         <v>13545909750.548668</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>14819212824.570616</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <v>16172706688.913439</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <v>16819614956.469976</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="2">
         <v>17821519770.741165</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="2">
         <v>21820209720.085629</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="2">
         <v>22693018108.889053</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="2">
         <v>23911972695.901939</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="2">
         <v>28357519930.870903</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="2">
         <v>29491820728.105736</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3" s="2">
         <v>35530084303.933441</v>
       </c>
-      <c r="N3" s="3">
+      <c r="N3" s="2">
         <v>38653374832.799126</v>
       </c>
-      <c r="O3" s="3">
+      <c r="O3" s="2">
         <v>41429605318.09726</v>
       </c>
-      <c r="P3" s="3">
+      <c r="P3" s="2">
         <v>41429605318.09726</v>
       </c>
-      <c r="Q3" s="3">
+      <c r="Q3" s="2">
         <v>41429605318.09726</v>
       </c>
-      <c r="R3" s="3">
+      <c r="R3" s="2">
         <v>43859025623.070145</v>
       </c>
-      <c r="S3" s="3">
+      <c r="S3" s="2">
         <v>43859025623.070145</v>
       </c>
-      <c r="T3" s="3">
+      <c r="T3" s="2">
         <v>46565294400.521698</v>
       </c>
-      <c r="U3" s="3">
+      <c r="U3" s="2">
         <v>46565294400.521698</v>
       </c>
-      <c r="V3" s="3">
+      <c r="V3" s="2">
         <v>49063926823.614243</v>
       </c>
-      <c r="W3" s="3">
+      <c r="W3" s="2">
         <v>49063926823.614243</v>
       </c>
-      <c r="X3" s="3">
+      <c r="X3" s="2">
         <v>51215249339.896927</v>
       </c>
-      <c r="Y3" s="3">
+      <c r="Y3" s="2">
         <v>51215249339.896927</v>
       </c>
-      <c r="Z3" s="3">
+      <c r="Z3" s="2">
         <v>51215249339.896927</v>
       </c>
-      <c r="AA3" s="3">
+      <c r="AA3" s="2">
         <v>51215249339.896927</v>
       </c>
-      <c r="AB3" s="3">
+      <c r="AB3" s="2">
         <v>51215249339.896927</v>
       </c>
     </row>
@@ -1597,7 +1604,7 @@
       <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C6">

</xml_diff>

<commit_message>
wording change of some coefficients
</commit_message>
<xml_diff>
--- a/data/scenarios.xlsx
+++ b/data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b9f352ed9e5ec6ce/00_플랜잇_철강inputoutput연구/steel_iotable/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{84D30074-6CA2-9646-BF7A-0F0212785F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90EDCEDF-9F7E-694E-8ED3-E824D6A77DDF}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="13_ncr:1_{84D30074-6CA2-9646-BF7A-0F0212785F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EB854DB-FA5B-444A-BC35-5A2E387C0A39}"/>
   <bookViews>
-    <workbookView xWindow="-9700" yWindow="760" windowWidth="25720" windowHeight="16980" xr2:uid="{8A7290D0-0CEE-BE47-A4B5-AA6B65E25749}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" xr2:uid="{8A7290D0-0CEE-BE47-A4B5-AA6B65E25749}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
code_h aggregation & RAS
code_h aggregation & RAS
</commit_message>
<xml_diff>
--- a/data/scenarios.xlsx
+++ b/data/scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b9f352ed9e5ec6ce/00_플랜잇_철강inputoutput연구/steel_iotable/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="13_ncr:1_{84D30074-6CA2-9646-BF7A-0F0212785F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EB854DB-FA5B-444A-BC35-5A2E387C0A39}"/>
+  <xr:revisionPtr revIDLastSave="108" documentId="13_ncr:1_{84D30074-6CA2-9646-BF7A-0F0212785F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{696157B1-82BA-3840-8612-8253AFBD28AE}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" xr2:uid="{8A7290D0-0CEE-BE47-A4B5-AA6B65E25749}"/>
   </bookViews>
@@ -664,82 +664,82 @@
         <v>9</v>
       </c>
       <c r="C3" s="2">
-        <v>13545909.750548668</v>
+        <v>966657.03881434398</v>
       </c>
       <c r="D3" s="2">
-        <v>14819212.824570615</v>
+        <v>2467521.2518916139</v>
       </c>
       <c r="E3" s="2">
-        <v>16172706.688913438</v>
+        <v>4086906.9687214158</v>
       </c>
       <c r="F3" s="2">
-        <v>16819614.956469975</v>
+        <v>4250383.2474702718</v>
       </c>
       <c r="G3" s="2">
-        <v>17821519.770741165</v>
+        <v>5078308.5278538484</v>
       </c>
       <c r="H3" s="2">
-        <v>21820209.720085628</v>
+        <v>11234183.3223552</v>
       </c>
       <c r="I3" s="2">
-        <v>22693018.108889055</v>
+        <v>11683550.655249387</v>
       </c>
       <c r="J3" s="2">
-        <v>23911972.695901938</v>
+        <v>12462126.544116681</v>
       </c>
       <c r="K3" s="2">
-        <v>28357519.930870902</v>
+        <v>18488000.976255953</v>
       </c>
       <c r="L3" s="2">
-        <v>29491820.728105735</v>
+        <v>19227521.01530619</v>
       </c>
       <c r="M3" s="2">
-        <v>35530084.303933442</v>
+        <v>26406961.963692084</v>
       </c>
       <c r="N3" s="2">
-        <v>38653374.832799129</v>
+        <v>31362092.688787885</v>
       </c>
       <c r="O3" s="2">
-        <v>41429605.318097256</v>
+        <v>35739728.489622861</v>
       </c>
       <c r="P3" s="2">
-        <v>41429605.318097256</v>
+        <v>35739728.489622861</v>
       </c>
       <c r="Q3" s="2">
-        <v>41429605.318097256</v>
+        <v>35739728.489622861</v>
       </c>
       <c r="R3" s="2">
-        <v>43859025.623070143</v>
+        <v>39575033.537424251</v>
       </c>
       <c r="S3" s="2">
-        <v>43859025.623070143</v>
+        <v>39575033.537424251</v>
       </c>
       <c r="T3" s="2">
-        <v>46565294.400521696</v>
+        <v>43833051.675945982</v>
       </c>
       <c r="U3" s="2">
-        <v>46565294.400521696</v>
+        <v>43833051.675945982</v>
       </c>
       <c r="V3" s="2">
-        <v>49063926.82361424</v>
+        <v>47807397.905829579</v>
       </c>
       <c r="W3" s="2">
-        <v>49063926.82361424</v>
+        <v>47807397.905829579</v>
       </c>
       <c r="X3" s="2">
-        <v>51215249.339896925</v>
+        <v>51215249.339896932</v>
       </c>
       <c r="Y3" s="2">
-        <v>51215249.339896925</v>
+        <v>51215249.339896932</v>
       </c>
       <c r="Z3" s="2">
-        <v>51215249.339896925</v>
+        <v>51215249.339896932</v>
       </c>
       <c r="AA3" s="2">
-        <v>51215249.339896925</v>
+        <v>51215249.339896932</v>
       </c>
       <c r="AB3" s="2">
-        <v>51215249.339896925</v>
+        <v>51215249.339896932</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.2">
@@ -836,82 +836,108 @@
         <v>5</v>
       </c>
       <c r="C5">
+        <f>h2portion!C6*h2portion!C3</f>
         <v>0</v>
       </c>
       <c r="D5">
+        <f>h2portion!D6*h2portion!D3</f>
         <v>0</v>
       </c>
       <c r="E5">
+        <f>h2portion!E6*h2portion!E3</f>
         <v>0</v>
       </c>
       <c r="F5">
+        <f>h2portion!F6*h2portion!F3</f>
         <v>0</v>
       </c>
       <c r="G5">
+        <f>h2portion!G6*h2portion!G3</f>
         <v>0</v>
       </c>
       <c r="H5">
-        <v>517553.6940288</v>
+        <f>h2portion!H6*h2portion!H3</f>
+        <v>517553.69402880006</v>
       </c>
       <c r="I5">
-        <v>412167.35183295468</v>
+        <f>h2portion!I6*h2portion!I3</f>
+        <v>412167.35183295474</v>
       </c>
       <c r="J5">
-        <v>560146.92785662669</v>
+        <f>h2portion!J6*h2portion!J3</f>
+        <v>560146.92785662657</v>
       </c>
       <c r="K5">
+        <f>h2portion!K6*h2portion!K3</f>
         <v>916125.71129999997</v>
       </c>
       <c r="L5">
+        <f>h2portion!L6*h2portion!L3</f>
         <v>910610.96129999997</v>
       </c>
       <c r="M5">
+        <f>h2portion!M6*h2portion!M3</f>
         <v>1365296.6420999998</v>
       </c>
       <c r="N5">
+        <f>h2portion!N6*h2portion!N3</f>
         <v>1642420.9049999998</v>
       </c>
       <c r="O5">
+        <f>h2portion!O6*h2portion!O3</f>
         <v>1784041.2501999999</v>
       </c>
       <c r="P5">
+        <f>h2portion!P6*h2portion!P3</f>
         <v>1706935.2497999999</v>
       </c>
       <c r="Q5">
+        <f>h2portion!Q6*h2portion!Q3</f>
         <v>1633362.2497999999</v>
       </c>
       <c r="R5">
-        <v>1751999.0734999997</v>
+        <f>h2portion!R6*h2portion!R3</f>
+        <v>1751999.0734999999</v>
       </c>
       <c r="S5">
-        <v>1696500</v>
+        <f>h2portion!S6*h2portion!S3</f>
+        <v>1696499.9999999998</v>
       </c>
       <c r="T5">
-        <v>1819062.80556</v>
+        <f>h2portion!T6*h2portion!T3</f>
+        <v>1819062.8055599998</v>
       </c>
       <c r="U5">
+        <f>h2portion!U6*h2portion!U3</f>
         <v>1741739.9999999998</v>
       </c>
       <c r="V5">
-        <v>1832800.1159999997</v>
+        <f>h2portion!V6*h2portion!V3</f>
+        <v>1832800.1159999999</v>
       </c>
       <c r="W5">
+        <f>h2portion!W6*h2portion!W3</f>
         <v>1755370.1159999995</v>
       </c>
       <c r="X5">
+        <f>h2portion!X6*h2portion!X3</f>
         <v>1811730.1749899995</v>
       </c>
       <c r="Y5">
+        <f>h2portion!Y6*h2portion!Y3</f>
         <v>1735173.6749999998</v>
       </c>
       <c r="Z5">
+        <f>h2portion!Z6*h2portion!Z3</f>
         <v>1662054.5249999999</v>
       </c>
       <c r="AA5">
-        <v>1592060.0000100001</v>
+        <f>h2portion!AA6*h2portion!AA3</f>
+        <v>1592060.0000099998</v>
       </c>
       <c r="AB5">
-        <v>1525190.4750000001</v>
+        <f>h2portion!AB6*h2portion!AB3</f>
+        <v>1525190.4749999999</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -922,82 +948,108 @@
         <v>6</v>
       </c>
       <c r="C6">
+        <f>h2portion!C6*h2portion!C4</f>
         <v>0</v>
       </c>
       <c r="D6">
+        <f>h2portion!D6*h2portion!D4</f>
         <v>0</v>
       </c>
       <c r="E6">
+        <f>h2portion!E6*h2portion!E4</f>
         <v>0</v>
       </c>
       <c r="F6">
+        <f>h2portion!F6*h2portion!F4</f>
         <v>0</v>
       </c>
       <c r="G6">
+        <f>h2portion!G6*h2portion!G4</f>
         <v>0</v>
       </c>
       <c r="H6">
+        <f>h2portion!H6*h2portion!H4</f>
         <v>557365.51664640009</v>
       </c>
       <c r="I6">
-        <v>522398.15523014031</v>
+        <f>h2portion!I6*h2portion!I4</f>
+        <v>522398.15523014037</v>
       </c>
       <c r="J6">
+        <f>h2portion!J6*h2portion!J4</f>
         <v>709953.66437642218</v>
       </c>
       <c r="K6">
+        <f>h2portion!K6*h2portion!K4</f>
         <v>1161136.07595</v>
       </c>
       <c r="L6">
+        <f>h2portion!L6*h2portion!L4</f>
         <v>1154146.45095</v>
       </c>
       <c r="M6">
-        <v>1730434.1161500001</v>
+        <f>h2portion!M6*h2portion!M4</f>
+        <v>1730434.1161499999</v>
       </c>
       <c r="N6">
+        <f>h2portion!N6*h2portion!N4</f>
         <v>2081673.0075000001</v>
       </c>
       <c r="O6">
-        <v>2261168.5613000002</v>
+        <f>h2portion!O6*h2portion!O4</f>
+        <v>2261168.5612999997</v>
       </c>
       <c r="P6">
-        <v>2163441.1886999998</v>
+        <f>h2portion!P6*h2portion!P4</f>
+        <v>2163441.1887000003</v>
       </c>
       <c r="Q6">
+        <f>h2portion!Q6*h2portion!Q4</f>
         <v>2070191.6887000001</v>
       </c>
       <c r="R6">
+        <f>h2portion!R6*h2portion!R4</f>
         <v>2220556.9652499999</v>
       </c>
       <c r="S6">
+        <f>h2portion!S6*h2portion!S4</f>
         <v>1930500</v>
       </c>
       <c r="T6">
-        <v>2069968.0201200002</v>
+        <f>h2portion!T6*h2portion!T4</f>
+        <v>2069968.02012</v>
       </c>
       <c r="U6">
+        <f>h2portion!U6*h2portion!U4</f>
         <v>1981980</v>
       </c>
       <c r="V6">
+        <f>h2portion!V6*h2portion!V4</f>
         <v>2085600.132</v>
       </c>
       <c r="W6">
+        <f>h2portion!W6*h2portion!W4</f>
         <v>1997490.1319999998</v>
       </c>
       <c r="X6">
+        <f>h2portion!X6*h2portion!X4</f>
         <v>2061623.9922299997</v>
       </c>
       <c r="Y6">
+        <f>h2portion!Y6*h2portion!Y4</f>
         <v>1974507.9750000001</v>
       </c>
       <c r="Z6">
+        <f>h2portion!Z6*h2portion!Z4</f>
         <v>1891303.425</v>
       </c>
       <c r="AA6">
-        <v>1811654.4827699999</v>
+        <f>h2portion!AA6*h2portion!AA4</f>
+        <v>1811654.4827700001</v>
       </c>
       <c r="AB6">
-        <v>1735561.575</v>
+        <f>h2portion!AB6*h2portion!AB4</f>
+        <v>1735561.5750000002</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.2">
@@ -1023,67 +1075,67 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>2209556.1552768</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>2199823.4243177469</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2989621.3940254841</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>4889554.6684499998</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <v>4860121.2934499998</v>
+        <v>0</v>
       </c>
       <c r="M7">
-        <v>7286873.9386500008</v>
+        <v>0</v>
       </c>
       <c r="N7">
-        <v>8765944.1325000003</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <v>9521801.5563000012</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <v>9110270.6937000006</v>
+        <v>0</v>
       </c>
       <c r="Q7">
-        <v>8717596.1937000006</v>
+        <v>0</v>
       </c>
       <c r="R7">
-        <v>9350785.75275</v>
+        <v>0</v>
       </c>
       <c r="S7">
-        <v>8482500</v>
+        <v>0</v>
       </c>
       <c r="T7">
-        <v>9095314.0277999993</v>
+        <v>0</v>
       </c>
       <c r="U7">
-        <v>8708700</v>
+        <v>0</v>
       </c>
       <c r="V7">
-        <v>9164000.5800000001</v>
+        <v>0</v>
       </c>
       <c r="W7">
-        <v>8776850.5799999982</v>
+        <v>0</v>
       </c>
       <c r="X7">
-        <v>9058650.8749499992</v>
+        <v>0</v>
       </c>
       <c r="Y7">
-        <v>8675868.375</v>
+        <v>0</v>
       </c>
       <c r="Z7">
-        <v>8310272.625</v>
+        <v>0</v>
       </c>
       <c r="AA7">
-        <v>7960300.0000499999</v>
+        <v>0</v>
       </c>
       <c r="AB7">
-        <v>7625952.375</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
@@ -1720,67 +1772,67 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>4976477827.1999998</v>
+        <v>4976477.8272000011</v>
       </c>
       <c r="I6">
-        <v>4792643625.9645901</v>
+        <v>4792643.6259645903</v>
       </c>
       <c r="J6">
-        <v>6513336370.4258909</v>
+        <v>6513336.3704258911</v>
       </c>
       <c r="K6">
-        <v>10652624550</v>
+        <v>10652624.550000001</v>
       </c>
       <c r="L6">
-        <v>10588499550</v>
+        <v>10588499.550000001</v>
       </c>
       <c r="M6">
-        <v>15875542350</v>
+        <v>15875542.35</v>
       </c>
       <c r="N6">
-        <v>19097917500</v>
+        <v>19097917.5</v>
       </c>
       <c r="O6">
-        <v>20744665700</v>
+        <v>20744665.699999999</v>
       </c>
       <c r="P6">
-        <v>19848084300</v>
+        <v>19848084.300000001</v>
       </c>
       <c r="Q6">
-        <v>18992584300</v>
+        <v>18992584.300000001</v>
       </c>
       <c r="R6">
-        <v>20372082250</v>
+        <v>20372082.25</v>
       </c>
       <c r="S6">
-        <v>19500000000</v>
+        <v>19500000</v>
       </c>
       <c r="T6">
-        <v>20908767880</v>
+        <v>20908767.879999999</v>
       </c>
       <c r="U6">
-        <v>20020000000</v>
+        <v>20020000</v>
       </c>
       <c r="V6">
-        <v>21066668000</v>
+        <v>21066668</v>
       </c>
       <c r="W6">
-        <v>20176667999.999996</v>
+        <v>20176667.999999996</v>
       </c>
       <c r="X6">
-        <v>20824484769.999996</v>
+        <v>20824484.769999996</v>
       </c>
       <c r="Y6">
-        <v>19944525000</v>
+        <v>19944525</v>
       </c>
       <c r="Z6">
-        <v>19104075000</v>
+        <v>19104075</v>
       </c>
       <c r="AA6">
-        <v>18299540230</v>
+        <v>18299540.23</v>
       </c>
       <c r="AB6">
-        <v>17530925000</v>
+        <v>17530925</v>
       </c>
     </row>
   </sheetData>

</xml_diff>